<commit_message>
Added Demo For Week 10
</commit_message>
<xml_diff>
--- a/Docs/Nisharg_Post_Joining_Sheet_G2.xlsx
+++ b/Docs/Nisharg_Post_Joining_Sheet_G2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\NishargSoni-458\RKIT_TRAINING\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3E88DE8-154C-496D-9387-6DD9E2850723}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DD992D9-DA2D-4A30-B264-537D8679619C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="68">
   <si>
     <t>#</t>
   </si>
@@ -230,24 +230,6 @@
   </si>
   <si>
     <t>pg_dump/pg_restore, pg_basebackup; PITR basics</t>
-  </si>
-  <si>
-    <t>Task</t>
-  </si>
-  <si>
-    <t>Study of .NET Core</t>
-  </si>
-  <si>
-    <t>Made Demos For DI,Options,Routing</t>
-  </si>
-  <si>
-    <t>Made InventoryMgt Demo using all learned .NET Core Concepts</t>
-  </si>
-  <si>
-    <t>Other</t>
-  </si>
-  <si>
-    <t>Domm</t>
   </si>
 </sst>
 </file>
@@ -326,9 +308,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -337,6 +316,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -687,7 +669,7 @@
       <c r="E3" t="s">
         <v>9</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="F3" s="7" t="s">
         <v>10</v>
       </c>
     </row>
@@ -707,7 +689,7 @@
       <c r="E4" t="s">
         <v>12</v>
       </c>
-      <c r="F4" s="4"/>
+      <c r="F4" s="7"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5">
@@ -725,7 +707,7 @@
       <c r="E5" t="s">
         <v>13</v>
       </c>
-      <c r="F5" s="4"/>
+      <c r="F5" s="7"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6">
@@ -743,7 +725,7 @@
       <c r="E6" t="s">
         <v>15</v>
       </c>
-      <c r="F6" s="4"/>
+      <c r="F6" s="7"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7">
@@ -761,7 +743,7 @@
       <c r="E7" t="s">
         <v>19</v>
       </c>
-      <c r="F7" s="4"/>
+      <c r="F7" s="7"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8">
@@ -779,7 +761,7 @@
       <c r="E8" t="s">
         <v>22</v>
       </c>
-      <c r="F8" s="4"/>
+      <c r="F8" s="7"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9">
@@ -797,7 +779,7 @@
       <c r="E9" t="s">
         <v>25</v>
       </c>
-      <c r="F9" s="4"/>
+      <c r="F9" s="7"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10">
@@ -815,7 +797,7 @@
       <c r="E10" t="s">
         <v>28</v>
       </c>
-      <c r="F10" s="4"/>
+      <c r="F10" s="7"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11">
@@ -833,7 +815,7 @@
       <c r="E11" t="s">
         <v>32</v>
       </c>
-      <c r="F11" s="4"/>
+      <c r="F11" s="7"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12">
@@ -845,7 +827,7 @@
       <c r="E12" t="s">
         <v>34</v>
       </c>
-      <c r="F12" s="4"/>
+      <c r="F12" s="7"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="E14" s="3"/>
@@ -854,65 +836,40 @@
       <c r="E15" s="3"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C16" s="5">
-        <v>46035</v>
-      </c>
-      <c r="D16" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="E16" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="F16" s="7">
-        <v>4</v>
-      </c>
+      <c r="C16" s="4"/>
+      <c r="D16" s="5"/>
+      <c r="E16" s="6"/>
+      <c r="F16" s="6"/>
     </row>
     <row r="17" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C17" s="7"/>
-      <c r="D17" s="7"/>
-      <c r="E17" s="7"/>
-      <c r="F17" s="7"/>
+      <c r="C17" s="6"/>
+      <c r="D17" s="6"/>
+      <c r="E17" s="6"/>
+      <c r="F17" s="6"/>
     </row>
     <row r="18" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C18" s="7"/>
-      <c r="D18" s="7"/>
-      <c r="E18" s="7" t="s">
-        <v>70</v>
-      </c>
-      <c r="F18" s="7">
-        <v>3.5</v>
-      </c>
+      <c r="C18" s="6"/>
+      <c r="D18" s="6"/>
+      <c r="E18" s="6"/>
+      <c r="F18" s="6"/>
     </row>
     <row r="19" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C19" s="7"/>
-      <c r="D19" s="7"/>
-      <c r="E19" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="F19" s="7">
-        <v>1.5</v>
-      </c>
+      <c r="C19" s="6"/>
+      <c r="D19" s="6"/>
+      <c r="E19" s="6"/>
+      <c r="F19" s="6"/>
     </row>
     <row r="20" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C20" s="7"/>
-      <c r="D20" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="E20" s="7" t="s">
-        <v>73</v>
-      </c>
-      <c r="F20" s="7">
-        <v>0.25</v>
-      </c>
+      <c r="C20" s="6"/>
+      <c r="D20" s="5"/>
+      <c r="E20" s="6"/>
+      <c r="F20" s="6"/>
     </row>
     <row r="21" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C21" s="7"/>
-      <c r="D21" s="7"/>
-      <c r="E21" s="7"/>
-      <c r="F21" s="7">
-        <f>SUM(F16:F20)</f>
-        <v>9.25</v>
-      </c>
+      <c r="C21" s="6"/>
+      <c r="D21" s="6"/>
+      <c r="E21" s="6"/>
+      <c r="F21" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1178,9 +1135,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1322,19 +1282,15 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EEA6786B-8A42-4A0D-80B4-9DE5209F0E64}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{43B1235E-D1DD-4EED-93B5-5B38ADCC7F24}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -1358,9 +1314,10 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{43B1235E-D1DD-4EED-93B5-5B38ADCC7F24}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EEA6786B-8A42-4A0D-80B4-9DE5209F0E64}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Added .net core demo
</commit_message>
<xml_diff>
--- a/Docs/Nisharg_Post_Joining_Sheet_G2.xlsx
+++ b/Docs/Nisharg_Post_Joining_Sheet_G2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\NishargSoni-458\RKIT_TRAINING\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5558B68-DFFC-463F-8063-4B7B14742B7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97B22A4E-9EDF-4B53-96F0-7DF414346E60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1273,18 +1273,18 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1306,18 +1306,18 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{43B1235E-D1DD-4EED-93B5-5B38ADCC7F24}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EEA6786B-8A42-4A0D-80B4-9DE5209F0E64}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{43B1235E-D1DD-4EED-93B5-5B38ADCC7F24}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>